<commit_message>
Item #43: add Pipeline Depth field to Intake Template
New Section B field on the Overview tab (Just Requirements | Up to
Design | Up to Implementation | Up to Deployment; blank defaults to
Up to Deployment). Styling copied from the Request Type row to match
the existing yellow-cell input convention. Instructions tab documents
the new field and the version line bumps to v1.1.

This is part 1/6 of Item #43 (Configurable Pipeline Depth) -- the
requester-facing input; downstream parsing/enforcement lands in
follow-up commits.
</commit_message>
<xml_diff>
--- a/docs/Templates/Intake Template.xlsx
+++ b/docs/Templates/Intake Template.xlsx
@@ -581,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="21" min="1" max="1"/>
@@ -649,85 +649,97 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="69.75" customHeight="1" s="22">
+    <row r="10" ht="55.5" customHeight="1" s="22">
       <c r="B10" s="25" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Pipeline Depth field</t>
+        </is>
+      </c>
+      <c r="C10" s="26" t="inlineStr">
+        <is>
+          <t>New in Section B. Tells FORGE how far to run this request: Just Requirements | Up to Design | Up to Implementation | Up to Deployment. Leave blank for the default (Up to Deployment, i.e. the full pipeline). This is a floor, not a menu -- "Up to Design" always runs Requirements and Design first, in that order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="22">
+      <c r="B11" s="25" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Requirements tab</t>
         </is>
       </c>
-      <c r="C10" s="26" t="inlineStr">
+      <c r="C11" s="26" t="inlineStr">
         <is>
           <t>Add one row per requirement. Use plain language — FORGE will convert these into properly structured user stories. Mark each row as Functional or Non-Functional and assign a priority. The Acceptance Criteria column is the most important: be specific about what 'done' looks like.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="22"/>
-    <row r="12" ht="18" customHeight="1" s="22">
-      <c r="B12" s="27" t="inlineStr">
+    <row r="12" ht="18" customHeight="1" s="22"/>
+    <row r="13" ht="15" customHeight="1" s="22">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>Colour guide</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="22">
-      <c r="B13" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Yellow cells</t>
-        </is>
-      </c>
-      <c r="C13" s="26" t="inlineStr">
-        <is>
-          <t>Fill these in. These are your input fields.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="22">
       <c r="B14" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Grey cells</t>
+          <t xml:space="preserve">  Yellow cells</t>
         </is>
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t>Do not edit. These are labels or calculated fields.</t>
+          <t>Fill these in. These are your input fields.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="22">
       <c r="B15" s="25" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Grey cells</t>
+        </is>
+      </c>
+      <c r="C15" s="26" t="inlineStr">
+        <is>
+          <t>Do not edit. These are labels or calculated fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="22">
+      <c r="B16" s="25" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Blue headers</t>
         </is>
       </c>
-      <c r="C15" s="26" t="inlineStr">
+      <c r="C16" s="26" t="inlineStr">
         <is>
           <t>Section titles. Do not edit.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="22"/>
-    <row r="17" ht="55.5" customHeight="1" s="22">
-      <c r="B17" s="25" t="inlineStr">
+    <row r="17" ht="55.5" customHeight="1" s="22"/>
+    <row r="18" ht="15" customHeight="1" s="22">
+      <c r="B18" s="25" t="inlineStr">
         <is>
           <t>Need help?</t>
         </is>
       </c>
-      <c r="C17" s="26" t="inlineStr">
+      <c r="C18" s="26" t="inlineStr">
         <is>
           <t>Contact your Orchestration Manager if you're unsure how to describe a requirement, or if you're not sure whether something is Functional or Non-Functional. It's better to ask than to leave a field blank.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="22"/>
-    <row r="19" ht="15" customHeight="1" s="22">
-      <c r="B19" s="25" t="inlineStr">
+    <row r="19" ht="15" customHeight="1" s="22"/>
+    <row r="20">
+      <c r="B20" s="25" t="inlineStr">
         <is>
           <t>Version</t>
         </is>
       </c>
-      <c r="C19" s="26" t="inlineStr">
-        <is>
-          <t>FORGE Intake Template v1.0  |  2026-07</t>
+      <c r="C20" s="26" t="inlineStr">
+        <is>
+          <t>FORGE Intake Template v1.1  |  2026-09-02  (Item #43: added Pipeline Depth field)</t>
         </is>
       </c>
     </row>
@@ -751,7 +763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="21" min="1" max="1"/>
@@ -874,218 +886,234 @@
     <row r="13" ht="27.75" customHeight="1" s="22">
       <c r="B13" s="28" t="inlineStr">
         <is>
-          <t>If Enhancement — Existing Service Name</t>
+          <t>Pipeline Depth</t>
         </is>
       </c>
       <c r="C13" s="29" t="inlineStr">
         <is>
-          <t>[Example: REQ-2026-03  (the exact folder name under services/ in the monorepo -- this request's own Request ID, not a descriptive name like client-portal)]</t>
+          <t>[Example: Just Requirements  |  Up to Design  |  Up to Implementation  |  Up to Deployment  (choose one; leave blank for Up to Deployment)]</t>
         </is>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" s="22">
       <c r="B14" s="28" t="inlineStr">
         <is>
+          <t>If Enhancement — Existing Service Name</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>[Example: REQ-2026-03  (the exact folder name under services/ in the monorepo -- this request's own Request ID, not a descriptive name like client-portal)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="28" t="inlineStr">
+        <is>
           <t>If Enhancement — Brief description of what exists today</t>
         </is>
       </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
         <is>
           <t>[Example: The portal lets clients view case status. There is no document upload.]</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="19.5" customHeight="1" s="22">
-      <c r="A16" s="27" t="inlineStr">
+    <row r="16" ht="19.5" customHeight="1" s="22"/>
+    <row r="17" ht="55.5" customHeight="1" s="22">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>C — Problem &amp; Purpose</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="55.5" customHeight="1" s="22">
-      <c r="B17" s="28" t="inlineStr">
-        <is>
-          <t>Problem being solved</t>
-        </is>
-      </c>
-      <c r="C17" s="29" t="inlineStr">
-        <is>
-          <t>[Example: Clients currently fax or mail documents to their lawyer. This creates delays and is unreliable. We need a way for clients to upload documents directly.]</t>
         </is>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" s="22">
       <c r="B18" s="28" t="inlineStr">
         <is>
-          <t>Purpose / Goal</t>
+          <t>Problem being solved</t>
         </is>
       </c>
       <c r="C18" s="29" t="inlineStr">
         <is>
-          <t>[Example: Allow clients to securely upload documents through the portal so lawyers receive them immediately without manual handling.]</t>
+          <t>[Example: Clients currently fax or mail documents to their lawyer. This creates delays and is unreliable. We need a way for clients to upload documents directly.]</t>
         </is>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" s="22">
       <c r="B19" s="28" t="inlineStr">
         <is>
-          <t>Who will use this? (Audience)</t>
+          <t>Purpose / Goal</t>
         </is>
       </c>
       <c r="C19" s="29" t="inlineStr">
         <is>
-          <t>[Example: Legal Aid Alberta clients (non-technical, using a web browser on phone or desktop). Internal staff will not use this feature directly.]</t>
+          <t>[Example: Allow clients to securely upload documents through the portal so lawyers receive them immediately without manual handling.]</t>
         </is>
       </c>
     </row>
     <row r="20" ht="27.75" customHeight="1" s="22">
       <c r="B20" s="28" t="inlineStr">
         <is>
+          <t>Who will use this? (Audience)</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>[Example: Legal Aid Alberta clients (non-technical, using a web browser on phone or desktop). Internal staff will not use this feature directly.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="28" t="inlineStr">
+        <is>
           <t>Approximate number of users / volume</t>
         </is>
       </c>
-      <c r="C20" s="29" t="inlineStr">
+      <c r="C21" s="29" t="inlineStr">
         <is>
           <t>[Example: ~500 clients/month uploading 1–3 documents each]</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="19.5" customHeight="1" s="22">
-      <c r="A22" s="27" t="inlineStr">
+    <row r="22" ht="19.5" customHeight="1" s="22"/>
+    <row r="23" ht="55.5" customHeight="1" s="22">
+      <c r="A23" s="27" t="inlineStr">
         <is>
           <t>D — Success Criteria &amp; Scope</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="55.5" customHeight="1" s="22">
-      <c r="B23" s="28" t="inlineStr">
-        <is>
-          <t>What does success look like?</t>
-        </is>
-      </c>
-      <c r="C23" s="29" t="inlineStr">
-        <is>
-          <t>[Example: A client can log in, select their case, upload a PDF or image, and their lawyer is notified within 5 minutes. Zero documents lost.]</t>
         </is>
       </c>
     </row>
     <row r="24" ht="55.5" customHeight="1" s="22">
       <c r="B24" s="28" t="inlineStr">
         <is>
-          <t>What is explicitly OUT of scope?</t>
+          <t>What does success look like?</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
         <is>
-          <t>[Example: E-signatures, document editing, automatic virus scanning (handled by infra team separately), integration with document management system (future phase).]</t>
+          <t>[Example: A client can log in, select their case, upload a PDF or image, and their lawyer is notified within 5 minutes. Zero documents lost.]</t>
         </is>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" s="22">
       <c r="B25" s="28" t="inlineStr">
         <is>
+          <t>What is explicitly OUT of scope?</t>
+        </is>
+      </c>
+      <c r="C25" s="29" t="inlineStr">
+        <is>
+          <t>[Example: E-signatures, document editing, automatic virus scanning (handled by infra team separately), integration with document management system (future phase).]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="28" t="inlineStr">
+        <is>
           <t>Are there related requests or dependencies?</t>
         </is>
       </c>
-      <c r="C25" s="29" t="inlineStr">
+      <c r="C26" s="29" t="inlineStr">
         <is>
           <t>[Example: Depends on the authentication upgrade (FORGE-2026-000) being deployed first.]</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="19.5" customHeight="1" s="22">
-      <c r="A27" s="27" t="inlineStr">
+    <row r="27" ht="19.5" customHeight="1" s="22"/>
+    <row r="28" ht="27.75" customHeight="1" s="22">
+      <c r="A28" s="27" t="inlineStr">
         <is>
           <t>E — Constraints &amp; Considerations</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="27.75" customHeight="1" s="22">
-      <c r="B28" s="28" t="inlineStr">
-        <is>
-          <t>Target completion date (if any)</t>
-        </is>
-      </c>
-      <c r="C28" s="29" t="inlineStr">
-        <is>
-          <t>[Example: 2026-09-30  (or: No hard deadline)]</t>
         </is>
       </c>
     </row>
     <row r="29" ht="42" customHeight="1" s="22">
       <c r="B29" s="28" t="inlineStr">
         <is>
-          <t>Regulatory or compliance constraints</t>
+          <t>Target completion date (if any)</t>
         </is>
       </c>
       <c r="C29" s="29" t="inlineStr">
         <is>
-          <t>[Example: Documents may contain client confidential information — must be encrypted at rest and in transit. Access logged.]</t>
+          <t>[Example: 2026-09-30  (or: No hard deadline)]</t>
         </is>
       </c>
     </row>
     <row r="30" ht="42" customHeight="1" s="22">
       <c r="B30" s="28" t="inlineStr">
         <is>
-          <t>Known technical constraints</t>
+          <t>Regulatory or compliance constraints</t>
         </is>
       </c>
       <c r="C30" s="29" t="inlineStr">
         <is>
-          <t>[Example: Must integrate with existing Azure Active Directory SSO. Max upload size 20 MB.]</t>
+          <t>[Example: Documents may contain client confidential information — must be encrypted at rest and in transit. Access logged.]</t>
         </is>
       </c>
     </row>
     <row r="31" ht="42" customHeight="1" s="22">
       <c r="B31" s="28" t="inlineStr">
         <is>
+          <t>Known technical constraints</t>
+        </is>
+      </c>
+      <c r="C31" s="29" t="inlineStr">
+        <is>
+          <t>[Example: Must integrate with existing Azure Active Directory SSO. Max upload size 20 MB.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="28" t="inlineStr">
+        <is>
           <t>Preferred tech / existing patterns to follow</t>
         </is>
       </c>
-      <c r="C31" s="29" t="inlineStr">
+      <c r="C32" s="29" t="inlineStr">
         <is>
           <t>[Example: Follow the same React component style as the existing portal. No new component libraries — use what is already in the project.]</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="19.5" customHeight="1" s="22">
-      <c r="A33" s="27" t="inlineStr">
+    <row r="33" ht="19.5" customHeight="1" s="22"/>
+    <row r="34" ht="42" customHeight="1" s="22">
+      <c r="A34" s="27" t="inlineStr">
         <is>
           <t>F — Additional Context</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="42" customHeight="1" s="22">
-      <c r="B34" s="28" t="inlineStr">
-        <is>
-          <t>Background / history the agent should know</t>
-        </is>
-      </c>
-      <c r="C34" s="29" t="inlineStr">
-        <is>
-          <t>[Example: This was requested after a client complaint in Q1 2026. The legal team has been asking for this for 18 months.]</t>
         </is>
       </c>
     </row>
     <row r="35" ht="27.75" customHeight="1" s="22">
       <c r="B35" s="28" t="inlineStr">
         <is>
-          <t>Links to supporting documents (SharePoint, Confluence, etc.)</t>
+          <t>Background / history the agent should know</t>
         </is>
       </c>
       <c r="C35" s="29" t="inlineStr">
         <is>
-          <t>[Example: https://legalaid.sharepoint.com/.../client-portal-doc-upload-brief.docx]</t>
+          <t>[Example: This was requested after a client complaint in Q1 2026. The legal team has been asking for this for 18 months.]</t>
         </is>
       </c>
     </row>
     <row r="36" ht="27.75" customHeight="1" s="22">
       <c r="B36" s="28" t="inlineStr">
         <is>
+          <t>Links to supporting documents (SharePoint, Confluence, etc.)</t>
+        </is>
+      </c>
+      <c r="C36" s="29" t="inlineStr">
+        <is>
+          <t>[Example: https://legalaid.sharepoint.com/.../client-portal-doc-upload-brief.docx]</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="28" t="inlineStr">
+        <is>
           <t>Anything else the Intake Agent should know</t>
         </is>
       </c>
-      <c r="C36" s="29" t="inlineStr">
+      <c r="C37" s="29" t="inlineStr">
         <is>
           <t>[Example: The stakeholder has a hard deadline driven by a board presentation on Oct 1.]</t>
         </is>

</xml_diff>